<commit_message>
added animations , a lot of animations
</commit_message>
<xml_diff>
--- a/server/Task Assigining.xlsx
+++ b/server/Task Assigining.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -655,13 +655,13 @@
         <v>No deadline</v>
       </c>
       <c r="L6" t="str">
-        <v>Not completed</v>
+        <v>13/9/2026, 3:25:14 pm</v>
       </c>
       <c r="M6" t="str">
-        <v>Ongoing</v>
+        <v>Completed</v>
       </c>
       <c r="N6" t="str">
-        <v>Ongoing</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="7">
@@ -833,13 +833,13 @@
         <v>10/9/2026, 3:17:00 am</v>
       </c>
       <c r="L10" t="str">
-        <v>Not completed</v>
+        <v>13/9/2026, 11:24:20 pm</v>
       </c>
       <c r="M10" t="str">
-        <v>Ongoing</v>
+        <v>Completed Late</v>
       </c>
       <c r="N10" t="str">
-        <v>Ongoing</v>
+        <v>No</v>
       </c>
     </row>
     <row r="11">
@@ -847,7 +847,7 @@
         <v>6a9d9f8b79f886cf3a661959</v>
       </c>
       <c r="B11" t="str">
-        <v>tryytyrry</v>
+        <v>(Deleted - Ongoing) tryytyrry</v>
       </c>
       <c r="C11" t="str">
         <v>tryytyrrytryytyrrytryytyrry</v>
@@ -877,18 +877,150 @@
         <v>12/9/2026, 10:44:00 pm</v>
       </c>
       <c r="L11" t="str">
-        <v>Not completed</v>
+        <v>Deleted on 7/9/2026, 12:17:24 am</v>
       </c>
       <c r="M11" t="str">
-        <v>Ongoing</v>
+        <v>Deleted (Ongoing)</v>
       </c>
       <c r="N11" t="str">
-        <v>Ongoing</v>
+        <v>Deleted (Ongoing)</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>6aa400457bdde79056e74ed5</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Complete you MyProfile Section !!!!!!!!!!!</v>
+      </c>
+      <c r="C12" t="str">
+        <v>from dropdown section, go to MyProfile and append your github link in link section and your skills in the about us section.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Core Team</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Gfg Supreme Account</v>
+      </c>
+      <c r="G12" t="str">
+        <v>geeksforgeeksbvp@gmail.com</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Aarti Singh</v>
+      </c>
+      <c r="I12" t="str">
+        <v>37aartisingh121212@gmail.com</v>
+      </c>
+      <c r="J12" t="str">
+        <v>11/9/2026, 6:51:09 pm</v>
+      </c>
+      <c r="K12" t="str">
+        <v>15/9/2026, 12:20:00 am</v>
+      </c>
+      <c r="L12" t="str">
+        <v>13/9/2026, 4:05:48 pm</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>6aa4008a7bdde79056e74f6c</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Complete you MyProfile Section !!!!!!!!!!!</v>
+      </c>
+      <c r="C13" t="str">
+        <v>from dropdown section, go to MyProfile and append your github link in link section and your skills in the about us section.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Social Media and Promotion</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Gfg Supreme Account</v>
+      </c>
+      <c r="G13" t="str">
+        <v>geeksforgeeksbvp@gmail.com</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Radhika Trivedi</v>
+      </c>
+      <c r="I13" t="str">
+        <v>radhikatriv0712@gmail.com</v>
+      </c>
+      <c r="J13" t="str">
+        <v>11/9/2026, 6:52:18 pm</v>
+      </c>
+      <c r="K13" t="str">
+        <v>No deadline</v>
+      </c>
+      <c r="L13" t="str">
+        <v>11/9/2026, 7:24:55 pm</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>6aa6edd472a52dafbea8e79a</v>
+      </c>
+      <c r="B14" t="str">
+        <v>(Deleted - Ongoing) test</v>
+      </c>
+      <c r="C14" t="str">
+        <v>this is text https://open.spotify.com hey</v>
+      </c>
+      <c r="D14" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Gfg Supreme Account</v>
+      </c>
+      <c r="G14" t="str">
+        <v>geeksforgeeksbvp@gmail.com</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Dev Malik</v>
+      </c>
+      <c r="I14" t="str">
+        <v>devmalik838400@gmail.com</v>
+      </c>
+      <c r="J14" t="str">
+        <v>14/9/2026, 12:09:16 am</v>
+      </c>
+      <c r="K14" t="str">
+        <v>No deadline</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Deleted on 14/9/2026, 12:09:48 am</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Deleted (Ongoing)</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Deleted (Ongoing)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>